<commit_message>
include product names - still needs testing
</commit_message>
<xml_diff>
--- a/reconcile/storage/input/vehicles_impute.xlsx
+++ b/reconcile/storage/input/vehicles_impute.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/benjamin_mcwilliams/Documents/bruegel/data_new/WORKING/INDUSTRY/tuone_v6/reconcile/storage/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFFD05D3-5EA7-E040-B604-A8F221F87DA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C08C08D-62ED-7047-9732-8C5250E04D2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="16660" xr2:uid="{BCDF9C02-A93F-4FDD-BCB7-C0839095CF07}"/>
   </bookViews>
@@ -161,31 +161,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C22" authorId="0" shapeId="0" xr:uid="{BB069DC0-8A6E-5949-BC1C-028E6717895D}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Ugne Keliauskaite:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Oxford</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="H24" authorId="0" shapeId="0" xr:uid="{145C7E98-B095-C643-8924-514EDD25BEC5}">
+    <comment ref="H23" authorId="0" shapeId="0" xr:uid="{145C7E98-B095-C643-8924-514EDD25BEC5}">
       <text>
         <r>
           <rPr>
@@ -218,7 +194,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I39" authorId="0" shapeId="0" xr:uid="{212D0BA5-2590-964B-94B4-A29484F5AA04}">
+    <comment ref="I38" authorId="0" shapeId="0" xr:uid="{212D0BA5-2590-964B-94B4-A29484F5AA04}">
       <text>
         <r>
           <rPr>
@@ -242,7 +218,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I68" authorId="0" shapeId="0" xr:uid="{A6DCB7E2-74E6-854F-8E16-ED35920E6252}">
+    <comment ref="I67" authorId="0" shapeId="0" xr:uid="{A6DCB7E2-74E6-854F-8E16-ED35920E6252}">
       <text>
         <r>
           <rPr>
@@ -266,7 +242,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C87" authorId="0" shapeId="0" xr:uid="{39646029-FBAA-B440-B731-9434C73CE445}">
+    <comment ref="C86" authorId="0" shapeId="0" xr:uid="{39646029-FBAA-B440-B731-9434C73CE445}">
       <text>
         <r>
           <rPr>
@@ -290,7 +266,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E100" authorId="0" shapeId="0" xr:uid="{D8F4CA31-F91E-AF45-ADD2-443248F0B75A}">
+    <comment ref="E99" authorId="0" shapeId="0" xr:uid="{D8F4CA31-F91E-AF45-ADD2-443248F0B75A}">
       <text>
         <r>
           <rPr>
@@ -314,7 +290,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I100" authorId="0" shapeId="0" xr:uid="{348C7426-DCB9-3442-84D9-DE241977A6F5}">
+    <comment ref="I99" authorId="0" shapeId="0" xr:uid="{348C7426-DCB9-3442-84D9-DE241977A6F5}">
       <text>
         <r>
           <rPr>
@@ -1555,7 +1531,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3546" uniqueCount="1309">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3540" uniqueCount="1309">
   <si>
     <t>facility_id_readable</t>
   </si>
@@ -7222,10 +7198,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{412528DA-AF97-D649-A38F-E0F2FFD8069D}" name="Table1" displayName="Table1" ref="A1:I107" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
-  <autoFilter ref="A1:I107" xr:uid="{412528DA-AF97-D649-A38F-E0F2FFD8069D}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I107">
-    <sortCondition ref="A1:A107"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{412528DA-AF97-D649-A38F-E0F2FFD8069D}" name="Table1" displayName="Table1" ref="A1:I106" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
+  <autoFilter ref="A1:I106" xr:uid="{412528DA-AF97-D649-A38F-E0F2FFD8069D}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I106">
+    <sortCondition ref="A1:A106"/>
   </sortState>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{88F84DCB-9434-3D44-9E03-D4FD2CDBE33E}" name="company_name" dataDxfId="8"/>
@@ -7570,7 +7546,7 @@
   <sheetPr>
     <tabColor rgb="FFC00000"/>
   </sheetPr>
-  <dimension ref="A1:J108"/>
+  <dimension ref="A1:J107"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.5" bestFit="1" customWidth="1"/>
@@ -8145,17 +8121,17 @@
         <v>142</v>
       </c>
       <c r="D21" s="163" t="s">
-        <v>143</v>
+        <v>71</v>
       </c>
       <c r="E21" s="163" t="s">
         <v>61</v>
       </c>
       <c r="F21" s="341"/>
-      <c r="G21" s="164">
-        <v>43655</v>
-      </c>
-      <c r="H21" s="164">
-        <v>43655</v>
+      <c r="G21" s="339">
+        <v>45657</v>
+      </c>
+      <c r="H21" s="339">
+        <v>45657</v>
       </c>
       <c r="I21" s="124">
         <v>46387</v>
@@ -8167,23 +8143,29 @@
         <v>57</v>
       </c>
       <c r="B22" s="163" t="s">
-        <v>141</v>
+        <v>161</v>
       </c>
       <c r="C22" s="163" t="s">
-        <v>142</v>
+        <v>162</v>
       </c>
       <c r="D22" s="163" t="s">
-        <v>71</v>
+        <v>143</v>
       </c>
       <c r="E22" s="163" t="s">
-        <v>148</v>
+        <v>124</v>
       </c>
       <c r="F22" s="341" t="s">
-        <v>151</v>
-      </c>
-      <c r="G22" s="163"/>
-      <c r="H22" s="163"/>
-      <c r="I22" s="161"/>
+        <v>166</v>
+      </c>
+      <c r="G22" s="164">
+        <v>46022</v>
+      </c>
+      <c r="H22" s="164">
+        <v>46022</v>
+      </c>
+      <c r="I22" s="161">
+        <v>150000</v>
+      </c>
       <c r="J22" s="161"/>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
@@ -8191,57 +8173,55 @@
         <v>57</v>
       </c>
       <c r="B23" s="163" t="s">
-        <v>161</v>
+        <v>141</v>
       </c>
       <c r="C23" s="163" t="s">
-        <v>162</v>
+        <v>1142</v>
       </c>
       <c r="D23" s="163" t="s">
-        <v>143</v>
+        <v>60</v>
       </c>
       <c r="E23" s="163" t="s">
-        <v>124</v>
-      </c>
-      <c r="F23" s="341" t="s">
-        <v>166</v>
-      </c>
+        <v>61</v>
+      </c>
+      <c r="F23" s="342"/>
       <c r="G23" s="164">
-        <v>46022</v>
+        <v>45291</v>
       </c>
       <c r="H23" s="164">
-        <v>46022</v>
+        <v>45291</v>
       </c>
       <c r="I23" s="161">
-        <v>150000</v>
-      </c>
-      <c r="J23" s="161"/>
+        <v>1076</v>
+      </c>
+      <c r="J23" s="124"/>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A24" s="163" t="s">
-        <v>57</v>
+        <v>264</v>
       </c>
       <c r="B24" s="163" t="s">
-        <v>141</v>
+        <v>265</v>
       </c>
       <c r="C24" s="163" t="s">
-        <v>1142</v>
+        <v>266</v>
       </c>
       <c r="D24" s="163" t="s">
-        <v>60</v>
+        <v>143</v>
       </c>
       <c r="E24" s="163" t="s">
-        <v>61</v>
-      </c>
-      <c r="F24" s="342"/>
+        <v>267</v>
+      </c>
+      <c r="F24" s="341" t="s">
+        <v>270</v>
+      </c>
       <c r="G24" s="164">
-        <v>45291</v>
+        <v>43440</v>
       </c>
       <c r="H24" s="164">
-        <v>45291</v>
-      </c>
-      <c r="I24" s="161">
-        <v>1076</v>
-      </c>
+        <v>43440</v>
+      </c>
+      <c r="I24" s="161"/>
       <c r="J24" s="124"/>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
@@ -8249,27 +8229,29 @@
         <v>264</v>
       </c>
       <c r="B25" s="163" t="s">
-        <v>265</v>
+        <v>161</v>
       </c>
       <c r="C25" s="163" t="s">
-        <v>266</v>
+        <v>278</v>
       </c>
       <c r="D25" s="163" t="s">
-        <v>143</v>
+        <v>60</v>
       </c>
       <c r="E25" s="163" t="s">
-        <v>267</v>
+        <v>61</v>
       </c>
       <c r="F25" s="341" t="s">
-        <v>270</v>
+        <v>280</v>
       </c>
       <c r="G25" s="164">
-        <v>43440</v>
+        <v>42855</v>
       </c>
       <c r="H25" s="164">
-        <v>43440</v>
-      </c>
-      <c r="I25" s="161"/>
+        <v>42855</v>
+      </c>
+      <c r="I25" s="161">
+        <v>400</v>
+      </c>
       <c r="J25" s="124"/>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.2">
@@ -8283,70 +8265,62 @@
         <v>278</v>
       </c>
       <c r="D26" s="163" t="s">
-        <v>60</v>
+        <v>143</v>
       </c>
       <c r="E26" s="163" t="s">
-        <v>61</v>
+        <v>124</v>
       </c>
       <c r="F26" s="341" t="s">
-        <v>280</v>
-      </c>
-      <c r="G26" s="164">
-        <v>42855</v>
-      </c>
-      <c r="H26" s="164">
-        <v>42855</v>
-      </c>
+        <v>286</v>
+      </c>
+      <c r="G26" s="163"/>
+      <c r="H26" s="163"/>
       <c r="I26" s="161">
-        <v>400</v>
-      </c>
-      <c r="J26" s="124"/>
+        <v>150000</v>
+      </c>
+      <c r="J26" s="161"/>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A27" s="163" t="s">
-        <v>264</v>
-      </c>
-      <c r="B27" s="163" t="s">
-        <v>161</v>
-      </c>
-      <c r="C27" s="163" t="s">
-        <v>278</v>
-      </c>
-      <c r="D27" s="163" t="s">
+      <c r="A27" s="183" t="s">
+        <v>297</v>
+      </c>
+      <c r="B27" s="183" t="s">
+        <v>141</v>
+      </c>
+      <c r="C27" s="183" t="s">
+        <v>298</v>
+      </c>
+      <c r="D27" s="183" t="s">
         <v>143</v>
       </c>
-      <c r="E27" s="163" t="s">
-        <v>124</v>
+      <c r="E27" s="183" t="s">
+        <v>192</v>
       </c>
       <c r="F27" s="341" t="s">
-        <v>286</v>
+        <v>299</v>
       </c>
       <c r="G27" s="163"/>
       <c r="H27" s="163"/>
-      <c r="I27" s="161">
-        <v>150000</v>
-      </c>
+      <c r="I27" s="161"/>
       <c r="J27" s="161"/>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A28" s="183" t="s">
-        <v>297</v>
-      </c>
-      <c r="B28" s="183" t="s">
-        <v>141</v>
-      </c>
-      <c r="C28" s="183" t="s">
-        <v>298</v>
-      </c>
-      <c r="D28" s="183" t="s">
-        <v>143</v>
-      </c>
-      <c r="E28" s="183" t="s">
+      <c r="A28" s="163" t="s">
+        <v>308</v>
+      </c>
+      <c r="B28" s="163" t="s">
+        <v>58</v>
+      </c>
+      <c r="C28" s="163" t="s">
+        <v>309</v>
+      </c>
+      <c r="D28" s="163" t="s">
+        <v>214</v>
+      </c>
+      <c r="E28" s="163" t="s">
         <v>192</v>
       </c>
-      <c r="F28" s="341" t="s">
-        <v>299</v>
-      </c>
+      <c r="F28" s="341"/>
       <c r="G28" s="163"/>
       <c r="H28" s="163"/>
       <c r="I28" s="161"/>
@@ -8354,21 +8328,23 @@
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A29" s="163" t="s">
-        <v>308</v>
+        <v>334</v>
       </c>
       <c r="B29" s="163" t="s">
-        <v>58</v>
+        <v>335</v>
       </c>
       <c r="C29" s="163" t="s">
-        <v>309</v>
+        <v>336</v>
       </c>
       <c r="D29" s="163" t="s">
-        <v>214</v>
+        <v>143</v>
       </c>
       <c r="E29" s="163" t="s">
-        <v>192</v>
-      </c>
-      <c r="F29" s="341"/>
+        <v>148</v>
+      </c>
+      <c r="F29" s="341" t="s">
+        <v>337</v>
+      </c>
       <c r="G29" s="163"/>
       <c r="H29" s="163"/>
       <c r="I29" s="161"/>
@@ -8379,10 +8355,10 @@
         <v>334</v>
       </c>
       <c r="B30" s="163" t="s">
-        <v>335</v>
+        <v>58</v>
       </c>
       <c r="C30" s="163" t="s">
-        <v>336</v>
+        <v>349</v>
       </c>
       <c r="D30" s="163" t="s">
         <v>143</v>
@@ -8390,23 +8366,23 @@
       <c r="E30" s="163" t="s">
         <v>148</v>
       </c>
-      <c r="F30" s="341" t="s">
-        <v>337</v>
-      </c>
+      <c r="F30" s="341"/>
       <c r="G30" s="163"/>
       <c r="H30" s="163"/>
-      <c r="I30" s="161"/>
+      <c r="I30" s="161">
+        <v>30000</v>
+      </c>
       <c r="J30" s="161"/>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A31" s="163" t="s">
-        <v>334</v>
+        <v>356</v>
       </c>
       <c r="B31" s="163" t="s">
-        <v>58</v>
+        <v>357</v>
       </c>
       <c r="C31" s="163" t="s">
-        <v>349</v>
+        <v>358</v>
       </c>
       <c r="D31" s="163" t="s">
         <v>143</v>
@@ -8414,53 +8390,55 @@
       <c r="E31" s="163" t="s">
         <v>148</v>
       </c>
-      <c r="F31" s="341"/>
-      <c r="G31" s="163"/>
-      <c r="H31" s="163"/>
+      <c r="F31" s="341" t="s">
+        <v>362</v>
+      </c>
+      <c r="G31" s="164">
+        <v>46203</v>
+      </c>
+      <c r="H31" s="164">
+        <v>46203</v>
+      </c>
       <c r="I31" s="161">
-        <v>30000</v>
+        <v>150000</v>
       </c>
       <c r="J31" s="161"/>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A32" s="163" t="s">
-        <v>356</v>
+        <v>374</v>
       </c>
       <c r="B32" s="163" t="s">
-        <v>357</v>
+        <v>58</v>
       </c>
       <c r="C32" s="163" t="s">
-        <v>358</v>
+        <v>375</v>
       </c>
       <c r="D32" s="163" t="s">
         <v>143</v>
       </c>
       <c r="E32" s="163" t="s">
-        <v>148</v>
+        <v>61</v>
       </c>
       <c r="F32" s="341" t="s">
-        <v>362</v>
-      </c>
-      <c r="G32" s="164">
-        <v>46203</v>
-      </c>
-      <c r="H32" s="164">
-        <v>46203</v>
-      </c>
+        <v>377</v>
+      </c>
+      <c r="G32" s="163"/>
+      <c r="H32" s="163"/>
       <c r="I32" s="161">
-        <v>150000</v>
+        <v>100</v>
       </c>
       <c r="J32" s="161"/>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A33" s="163" t="s">
-        <v>374</v>
+        <v>385</v>
       </c>
       <c r="B33" s="163" t="s">
-        <v>58</v>
+        <v>182</v>
       </c>
       <c r="C33" s="163" t="s">
-        <v>375</v>
+        <v>386</v>
       </c>
       <c r="D33" s="163" t="s">
         <v>143</v>
@@ -8469,24 +8447,28 @@
         <v>61</v>
       </c>
       <c r="F33" s="341" t="s">
-        <v>377</v>
-      </c>
-      <c r="G33" s="163"/>
-      <c r="H33" s="163"/>
+        <v>387</v>
+      </c>
+      <c r="G33" s="164">
+        <v>46053</v>
+      </c>
+      <c r="H33" s="164">
+        <v>46053</v>
+      </c>
       <c r="I33" s="161">
-        <v>100</v>
+        <v>5591</v>
       </c>
       <c r="J33" s="161"/>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A34" s="163" t="s">
-        <v>385</v>
+        <v>399</v>
       </c>
       <c r="B34" s="163" t="s">
-        <v>182</v>
+        <v>58</v>
       </c>
       <c r="C34" s="163" t="s">
-        <v>386</v>
+        <v>401</v>
       </c>
       <c r="D34" s="163" t="s">
         <v>143</v>
@@ -8495,16 +8477,16 @@
         <v>61</v>
       </c>
       <c r="F34" s="341" t="s">
-        <v>387</v>
+        <v>405</v>
       </c>
       <c r="G34" s="164">
-        <v>46053</v>
+        <v>45447</v>
       </c>
       <c r="H34" s="164">
-        <v>46053</v>
-      </c>
-      <c r="I34" s="161">
-        <v>5591</v>
+        <v>45447</v>
+      </c>
+      <c r="I34" s="343">
+        <v>250000</v>
       </c>
       <c r="J34" s="161"/>
     </row>
@@ -8513,10 +8495,10 @@
         <v>399</v>
       </c>
       <c r="B35" s="163" t="s">
-        <v>58</v>
+        <v>318</v>
       </c>
       <c r="C35" s="163" t="s">
-        <v>401</v>
+        <v>414</v>
       </c>
       <c r="D35" s="163" t="s">
         <v>143</v>
@@ -8524,17 +8506,11 @@
       <c r="E35" s="163" t="s">
         <v>61</v>
       </c>
-      <c r="F35" s="341" t="s">
-        <v>405</v>
-      </c>
-      <c r="G35" s="164">
-        <v>45447</v>
-      </c>
-      <c r="H35" s="164">
-        <v>45447</v>
-      </c>
-      <c r="I35" s="343">
-        <v>250000</v>
+      <c r="F35" s="341"/>
+      <c r="G35" s="163"/>
+      <c r="H35" s="163"/>
+      <c r="I35" s="161">
+        <v>44286</v>
       </c>
       <c r="J35" s="161"/>
     </row>
@@ -8549,31 +8525,31 @@
         <v>414</v>
       </c>
       <c r="D36" s="163" t="s">
-        <v>143</v>
+        <v>71</v>
       </c>
       <c r="E36" s="163" t="s">
-        <v>61</v>
+        <v>148</v>
       </c>
       <c r="F36" s="341"/>
       <c r="G36" s="163"/>
       <c r="H36" s="163"/>
       <c r="I36" s="161">
-        <v>44286</v>
+        <v>300000</v>
       </c>
       <c r="J36" s="161"/>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A37" s="163" t="s">
-        <v>399</v>
+        <v>428</v>
       </c>
       <c r="B37" s="163" t="s">
-        <v>318</v>
+        <v>429</v>
       </c>
       <c r="C37" s="163" t="s">
-        <v>414</v>
+        <v>430</v>
       </c>
       <c r="D37" s="163" t="s">
-        <v>71</v>
+        <v>143</v>
       </c>
       <c r="E37" s="163" t="s">
         <v>148</v>
@@ -8581,42 +8557,47 @@
       <c r="F37" s="341"/>
       <c r="G37" s="163"/>
       <c r="H37" s="163"/>
-      <c r="I37" s="161">
-        <v>300000</v>
-      </c>
+      <c r="I37" s="161"/>
       <c r="J37" s="161"/>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A38" s="163" t="s">
-        <v>428</v>
+        <v>434</v>
       </c>
       <c r="B38" s="163" t="s">
-        <v>429</v>
+        <v>435</v>
       </c>
       <c r="C38" s="163" t="s">
-        <v>430</v>
+        <v>436</v>
       </c>
       <c r="D38" s="163" t="s">
         <v>143</v>
       </c>
       <c r="E38" s="163" t="s">
-        <v>148</v>
-      </c>
-      <c r="F38" s="341"/>
-      <c r="G38" s="163"/>
-      <c r="H38" s="163"/>
-      <c r="I38" s="161"/>
+        <v>61</v>
+      </c>
+      <c r="F38" s="342"/>
+      <c r="G38" s="126">
+        <v>43891</v>
+      </c>
+      <c r="H38" s="126">
+        <v>43891</v>
+      </c>
+      <c r="I38" s="124">
+        <f>28213+43839</f>
+        <v>72052</v>
+      </c>
       <c r="J38" s="161"/>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A39" s="163" t="s">
-        <v>434</v>
+        <v>443</v>
       </c>
       <c r="B39" s="163" t="s">
-        <v>435</v>
+        <v>444</v>
       </c>
       <c r="C39" s="163" t="s">
-        <v>436</v>
+        <v>445</v>
       </c>
       <c r="D39" s="163" t="s">
         <v>143</v>
@@ -8624,28 +8605,27 @@
       <c r="E39" s="163" t="s">
         <v>61</v>
       </c>
-      <c r="F39" s="342"/>
-      <c r="G39" s="126">
-        <v>43891</v>
-      </c>
+      <c r="F39" s="342">
+        <v>2020</v>
+      </c>
+      <c r="G39" s="126"/>
       <c r="H39" s="126">
-        <v>43891</v>
+        <v>45657</v>
       </c>
       <c r="I39" s="124">
-        <f>28213+43839</f>
-        <v>72052</v>
-      </c>
-      <c r="J39" s="161"/>
+        <v>37239</v>
+      </c>
+      <c r="J39" s="343"/>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A40" s="163" t="s">
-        <v>443</v>
+        <v>462</v>
       </c>
       <c r="B40" s="163" t="s">
-        <v>444</v>
+        <v>58</v>
       </c>
       <c r="C40" s="163" t="s">
-        <v>445</v>
+        <v>463</v>
       </c>
       <c r="D40" s="163" t="s">
         <v>143</v>
@@ -8654,16 +8634,18 @@
         <v>61</v>
       </c>
       <c r="F40" s="342">
-        <v>2020</v>
-      </c>
-      <c r="G40" s="126"/>
+        <v>2015</v>
+      </c>
+      <c r="G40" s="126">
+        <v>42005</v>
+      </c>
       <c r="H40" s="126">
-        <v>45657</v>
-      </c>
-      <c r="I40" s="124">
-        <v>37239</v>
-      </c>
-      <c r="J40" s="343"/>
+        <v>42005</v>
+      </c>
+      <c r="I40" s="343">
+        <v>18427</v>
+      </c>
+      <c r="J40" s="161"/>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A41" s="163" t="s">
@@ -8676,22 +8658,18 @@
         <v>463</v>
       </c>
       <c r="D41" s="163" t="s">
-        <v>143</v>
+        <v>71</v>
       </c>
       <c r="E41" s="163" t="s">
         <v>61</v>
       </c>
-      <c r="F41" s="342">
-        <v>2015</v>
-      </c>
-      <c r="G41" s="126">
-        <v>42005</v>
-      </c>
-      <c r="H41" s="126">
-        <v>42005</v>
-      </c>
+      <c r="F41" s="341">
+        <v>2019</v>
+      </c>
+      <c r="G41" s="163"/>
+      <c r="H41" s="163"/>
       <c r="I41" s="343">
-        <v>18427</v>
+        <v>2650</v>
       </c>
       <c r="J41" s="161"/>
     </row>
@@ -8711,15 +8689,13 @@
       <c r="E42" s="163" t="s">
         <v>61</v>
       </c>
-      <c r="F42" s="341">
-        <v>2019</v>
-      </c>
+      <c r="F42" s="341"/>
       <c r="G42" s="163"/>
       <c r="H42" s="163"/>
       <c r="I42" s="343">
-        <v>2650</v>
-      </c>
-      <c r="J42" s="161"/>
+        <v>73662.5</v>
+      </c>
+      <c r="J42" s="124"/>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A43" s="163" t="s">
@@ -8729,19 +8705,25 @@
         <v>58</v>
       </c>
       <c r="C43" s="163" t="s">
-        <v>463</v>
+        <v>477</v>
       </c>
       <c r="D43" s="163" t="s">
-        <v>71</v>
+        <v>143</v>
       </c>
       <c r="E43" s="163" t="s">
         <v>61</v>
       </c>
-      <c r="F43" s="341"/>
-      <c r="G43" s="163"/>
-      <c r="H43" s="163"/>
-      <c r="I43" s="343">
-        <v>73662.5</v>
+      <c r="F43" s="342">
+        <v>2020</v>
+      </c>
+      <c r="G43" s="126">
+        <v>43831</v>
+      </c>
+      <c r="H43" s="126">
+        <v>43831</v>
+      </c>
+      <c r="I43" s="161">
+        <v>4760</v>
       </c>
       <c r="J43" s="124"/>
     </row>
@@ -8756,23 +8738,19 @@
         <v>477</v>
       </c>
       <c r="D44" s="163" t="s">
-        <v>143</v>
+        <v>71</v>
       </c>
       <c r="E44" s="163" t="s">
         <v>61</v>
       </c>
-      <c r="F44" s="342">
-        <v>2020</v>
-      </c>
+      <c r="F44" s="342"/>
       <c r="G44" s="126">
-        <v>43831</v>
+        <v>45260</v>
       </c>
       <c r="H44" s="126">
-        <v>43831</v>
-      </c>
-      <c r="I44" s="161">
-        <v>4760</v>
-      </c>
+        <v>45261</v>
+      </c>
+      <c r="I44" s="124"/>
       <c r="J44" s="124"/>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.2">
@@ -8783,23 +8761,19 @@
         <v>58</v>
       </c>
       <c r="C45" s="163" t="s">
-        <v>477</v>
+        <v>485</v>
       </c>
       <c r="D45" s="163" t="s">
-        <v>71</v>
+        <v>143</v>
       </c>
       <c r="E45" s="163" t="s">
         <v>61</v>
       </c>
       <c r="F45" s="342"/>
-      <c r="G45" s="126">
-        <v>45260</v>
-      </c>
-      <c r="H45" s="126">
-        <v>45261</v>
-      </c>
+      <c r="G45" s="105"/>
+      <c r="H45" s="105"/>
       <c r="I45" s="124"/>
-      <c r="J45" s="124"/>
+      <c r="J45" s="343"/>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A46" s="163" t="s">
@@ -8809,7 +8783,7 @@
         <v>58</v>
       </c>
       <c r="C46" s="163" t="s">
-        <v>485</v>
+        <v>490</v>
       </c>
       <c r="D46" s="163" t="s">
         <v>143</v>
@@ -8817,10 +8791,18 @@
       <c r="E46" s="163" t="s">
         <v>61</v>
       </c>
-      <c r="F46" s="342"/>
-      <c r="G46" s="105"/>
-      <c r="H46" s="105"/>
-      <c r="I46" s="124"/>
+      <c r="F46" s="342">
+        <v>2018</v>
+      </c>
+      <c r="G46" s="126">
+        <v>43101</v>
+      </c>
+      <c r="H46" s="126">
+        <v>43102</v>
+      </c>
+      <c r="I46" s="124">
+        <v>83195</v>
+      </c>
       <c r="J46" s="343"/>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.2">
@@ -8831,7 +8813,7 @@
         <v>58</v>
       </c>
       <c r="C47" s="163" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="D47" s="163" t="s">
         <v>143</v>
@@ -8839,17 +8821,17 @@
       <c r="E47" s="163" t="s">
         <v>61</v>
       </c>
-      <c r="F47" s="342">
-        <v>2018</v>
-      </c>
-      <c r="G47" s="126">
-        <v>43101</v>
+      <c r="F47" s="341">
+        <v>2016</v>
+      </c>
+      <c r="G47" s="164">
+        <v>42370</v>
       </c>
       <c r="H47" s="126">
-        <v>43102</v>
+        <v>42370</v>
       </c>
       <c r="I47" s="124">
-        <v>83195</v>
+        <v>62577.5</v>
       </c>
       <c r="J47" s="343"/>
     </row>
@@ -8858,10 +8840,10 @@
         <v>462</v>
       </c>
       <c r="B48" s="163" t="s">
-        <v>58</v>
+        <v>318</v>
       </c>
       <c r="C48" s="163" t="s">
-        <v>492</v>
+        <v>496</v>
       </c>
       <c r="D48" s="163" t="s">
         <v>143</v>
@@ -8870,18 +8852,16 @@
         <v>61</v>
       </c>
       <c r="F48" s="341">
-        <v>2016</v>
+        <v>2019</v>
       </c>
       <c r="G48" s="164">
-        <v>42370</v>
-      </c>
-      <c r="H48" s="126">
-        <v>42370</v>
-      </c>
+        <v>43617</v>
+      </c>
+      <c r="H48" s="105"/>
       <c r="I48" s="124">
-        <v>62577.5</v>
-      </c>
-      <c r="J48" s="343"/>
+        <v>10739</v>
+      </c>
+      <c r="J48" s="161"/>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A49" s="163" t="s">
@@ -8894,43 +8874,35 @@
         <v>496</v>
       </c>
       <c r="D49" s="163" t="s">
-        <v>143</v>
+        <v>71</v>
       </c>
       <c r="E49" s="163" t="s">
-        <v>61</v>
-      </c>
-      <c r="F49" s="341">
-        <v>2019</v>
-      </c>
+        <v>124</v>
+      </c>
+      <c r="F49" s="341"/>
       <c r="G49" s="164">
-        <v>43617</v>
-      </c>
-      <c r="H49" s="105"/>
-      <c r="I49" s="124">
-        <v>10739</v>
-      </c>
-      <c r="J49" s="161"/>
+        <v>46539</v>
+      </c>
+      <c r="H49" s="163"/>
+      <c r="I49" s="161"/>
+      <c r="J49" s="124"/>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A50" s="163" t="s">
         <v>462</v>
       </c>
       <c r="B50" s="163" t="s">
-        <v>318</v>
+        <v>265</v>
       </c>
       <c r="C50" s="163" t="s">
-        <v>496</v>
-      </c>
-      <c r="D50" s="163" t="s">
-        <v>71</v>
-      </c>
+        <v>1138</v>
+      </c>
+      <c r="D50" s="163"/>
       <c r="E50" s="163" t="s">
-        <v>124</v>
+        <v>61</v>
       </c>
       <c r="F50" s="341"/>
-      <c r="G50" s="164">
-        <v>46539</v>
-      </c>
+      <c r="G50" s="164"/>
       <c r="H50" s="163"/>
       <c r="I50" s="161"/>
       <c r="J50" s="124"/>
@@ -8940,19 +8912,21 @@
         <v>462</v>
       </c>
       <c r="B51" s="163" t="s">
-        <v>265</v>
+        <v>357</v>
       </c>
       <c r="C51" s="163" t="s">
-        <v>1138</v>
-      </c>
-      <c r="D51" s="163"/>
+        <v>505</v>
+      </c>
+      <c r="D51" s="163" t="s">
+        <v>143</v>
+      </c>
       <c r="E51" s="163" t="s">
-        <v>61</v>
-      </c>
-      <c r="F51" s="341"/>
-      <c r="G51" s="164"/>
-      <c r="H51" s="163"/>
-      <c r="I51" s="161"/>
+        <v>148</v>
+      </c>
+      <c r="F51" s="342"/>
+      <c r="G51" s="105"/>
+      <c r="H51" s="105"/>
+      <c r="I51" s="124"/>
       <c r="J51" s="124"/>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.2">
@@ -8960,21 +8934,27 @@
         <v>462</v>
       </c>
       <c r="B52" s="163" t="s">
-        <v>357</v>
+        <v>161</v>
       </c>
       <c r="C52" s="163" t="s">
-        <v>505</v>
+        <v>510</v>
       </c>
       <c r="D52" s="163" t="s">
         <v>143</v>
       </c>
       <c r="E52" s="163" t="s">
-        <v>148</v>
-      </c>
-      <c r="F52" s="342"/>
-      <c r="G52" s="105"/>
-      <c r="H52" s="105"/>
-      <c r="I52" s="124"/>
+        <v>61</v>
+      </c>
+      <c r="F52" s="341" t="s">
+        <v>511</v>
+      </c>
+      <c r="G52" s="164">
+        <v>44530</v>
+      </c>
+      <c r="H52" s="163"/>
+      <c r="I52" s="124">
+        <v>50444</v>
+      </c>
       <c r="J52" s="124"/>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.2">
@@ -8988,48 +8968,48 @@
         <v>510</v>
       </c>
       <c r="D53" s="163" t="s">
-        <v>143</v>
+        <v>71</v>
       </c>
       <c r="E53" s="163" t="s">
-        <v>61</v>
+        <v>124</v>
       </c>
       <c r="F53" s="341" t="s">
-        <v>511</v>
+        <v>518</v>
       </c>
       <c r="G53" s="164">
-        <v>44530</v>
+        <v>46023</v>
       </c>
       <c r="H53" s="163"/>
-      <c r="I53" s="124">
-        <v>50444</v>
-      </c>
+      <c r="I53" s="161"/>
       <c r="J53" s="124"/>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A54" s="163" t="s">
-        <v>462</v>
+        <v>521</v>
       </c>
       <c r="B54" s="163" t="s">
-        <v>161</v>
+        <v>141</v>
       </c>
       <c r="C54" s="163" t="s">
-        <v>510</v>
+        <v>522</v>
       </c>
       <c r="D54" s="163" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="E54" s="163" t="s">
-        <v>124</v>
-      </c>
-      <c r="F54" s="341" t="s">
-        <v>518</v>
+        <v>61</v>
+      </c>
+      <c r="F54" s="341">
+        <v>2013</v>
       </c>
       <c r="G54" s="164">
-        <v>46023</v>
+        <v>41275</v>
       </c>
       <c r="H54" s="163"/>
-      <c r="I54" s="161"/>
-      <c r="J54" s="124"/>
+      <c r="I54" s="161">
+        <v>40710</v>
+      </c>
+      <c r="J54" s="161"/>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A55" s="163" t="s">
@@ -9042,46 +9022,44 @@
         <v>522</v>
       </c>
       <c r="D55" s="163" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="E55" s="163" t="s">
-        <v>61</v>
-      </c>
-      <c r="F55" s="341">
-        <v>2013</v>
-      </c>
-      <c r="G55" s="164">
-        <v>41275</v>
-      </c>
+        <v>124</v>
+      </c>
+      <c r="F55" s="341"/>
+      <c r="G55" s="163"/>
       <c r="H55" s="163"/>
       <c r="I55" s="161">
-        <v>40710</v>
+        <v>100000</v>
       </c>
       <c r="J55" s="161"/>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A56" s="163" t="s">
-        <v>521</v>
-      </c>
-      <c r="B56" s="163" t="s">
-        <v>141</v>
-      </c>
-      <c r="C56" s="163" t="s">
-        <v>522</v>
-      </c>
-      <c r="D56" s="163" t="s">
-        <v>71</v>
-      </c>
-      <c r="E56" s="163" t="s">
-        <v>124</v>
-      </c>
-      <c r="F56" s="341"/>
-      <c r="G56" s="163"/>
-      <c r="H56" s="163"/>
-      <c r="I56" s="161">
-        <v>100000</v>
-      </c>
-      <c r="J56" s="161"/>
+      <c r="A56" s="152" t="s">
+        <v>1063</v>
+      </c>
+      <c r="B56" s="152" t="s">
+        <v>265</v>
+      </c>
+      <c r="C56" s="152" t="s">
+        <v>1076</v>
+      </c>
+      <c r="D56" s="152" t="s">
+        <v>60</v>
+      </c>
+      <c r="E56" s="152" t="s">
+        <v>61</v>
+      </c>
+      <c r="F56" s="338"/>
+      <c r="G56" s="152"/>
+      <c r="H56" s="339">
+        <v>45657</v>
+      </c>
+      <c r="I56" s="337">
+        <v>16874</v>
+      </c>
+      <c r="J56" s="124"/>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A57" s="152" t="s">
@@ -9091,7 +9069,7 @@
         <v>265</v>
       </c>
       <c r="C57" s="152" t="s">
-        <v>1076</v>
+        <v>1134</v>
       </c>
       <c r="D57" s="152" t="s">
         <v>60</v>
@@ -9105,7 +9083,7 @@
         <v>45657</v>
       </c>
       <c r="I57" s="337">
-        <v>16874</v>
+        <v>2117</v>
       </c>
       <c r="J57" s="124"/>
     </row>
@@ -9117,7 +9095,7 @@
         <v>265</v>
       </c>
       <c r="C58" s="152" t="s">
-        <v>1134</v>
+        <v>1137</v>
       </c>
       <c r="D58" s="152" t="s">
         <v>60</v>
@@ -9128,12 +9106,12 @@
       <c r="F58" s="338"/>
       <c r="G58" s="152"/>
       <c r="H58" s="339">
-        <v>45657</v>
+        <v>45291</v>
       </c>
       <c r="I58" s="337">
-        <v>2117</v>
-      </c>
-      <c r="J58" s="124"/>
+        <v>18174</v>
+      </c>
+      <c r="J58" s="161"/>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A59" s="152" t="s">
@@ -9143,7 +9121,7 @@
         <v>265</v>
       </c>
       <c r="C59" s="152" t="s">
-        <v>1137</v>
+        <v>1133</v>
       </c>
       <c r="D59" s="152" t="s">
         <v>60</v>
@@ -9154,10 +9132,10 @@
       <c r="F59" s="338"/>
       <c r="G59" s="152"/>
       <c r="H59" s="339">
-        <v>45291</v>
+        <v>45657</v>
       </c>
       <c r="I59" s="337">
-        <v>18174</v>
+        <v>615</v>
       </c>
       <c r="J59" s="161"/>
     </row>
@@ -9169,7 +9147,7 @@
         <v>265</v>
       </c>
       <c r="C60" s="152" t="s">
-        <v>1133</v>
+        <v>1064</v>
       </c>
       <c r="D60" s="152" t="s">
         <v>60</v>
@@ -9179,37 +9157,35 @@
       </c>
       <c r="F60" s="338"/>
       <c r="G60" s="152"/>
-      <c r="H60" s="339">
+      <c r="H60" s="164">
         <v>45657</v>
       </c>
       <c r="I60" s="337">
-        <v>615</v>
+        <v>71051</v>
       </c>
       <c r="J60" s="161"/>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A61" s="152" t="s">
-        <v>1063</v>
-      </c>
-      <c r="B61" s="152" t="s">
-        <v>265</v>
-      </c>
-      <c r="C61" s="152" t="s">
-        <v>1064</v>
-      </c>
-      <c r="D61" s="152" t="s">
-        <v>60</v>
-      </c>
-      <c r="E61" s="152" t="s">
+      <c r="A61" s="163" t="s">
+        <v>541</v>
+      </c>
+      <c r="B61" s="163" t="s">
+        <v>542</v>
+      </c>
+      <c r="C61" s="163" t="s">
+        <v>543</v>
+      </c>
+      <c r="D61" s="163" t="s">
+        <v>143</v>
+      </c>
+      <c r="E61" s="163" t="s">
         <v>61</v>
       </c>
-      <c r="F61" s="338"/>
-      <c r="G61" s="152"/>
-      <c r="H61" s="164">
-        <v>45657</v>
-      </c>
-      <c r="I61" s="337">
-        <v>71051</v>
+      <c r="F61" s="341"/>
+      <c r="G61" s="163"/>
+      <c r="H61" s="163"/>
+      <c r="I61" s="161">
+        <v>26699</v>
       </c>
       <c r="J61" s="161"/>
     </row>
@@ -9224,43 +9200,47 @@
         <v>543</v>
       </c>
       <c r="D62" s="163" t="s">
-        <v>143</v>
+        <v>71</v>
       </c>
       <c r="E62" s="163" t="s">
-        <v>61</v>
-      </c>
-      <c r="F62" s="341"/>
-      <c r="G62" s="163"/>
-      <c r="H62" s="163"/>
-      <c r="I62" s="161">
-        <v>26699</v>
-      </c>
+        <v>148</v>
+      </c>
+      <c r="F62" s="341">
+        <v>2026</v>
+      </c>
+      <c r="G62" s="164">
+        <v>46203</v>
+      </c>
+      <c r="H62" s="164">
+        <v>46203</v>
+      </c>
+      <c r="I62" s="161"/>
       <c r="J62" s="161"/>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A63" s="163" t="s">
-        <v>541</v>
+        <v>561</v>
       </c>
       <c r="B63" s="163" t="s">
-        <v>542</v>
+        <v>429</v>
       </c>
       <c r="C63" s="163" t="s">
-        <v>543</v>
+        <v>562</v>
       </c>
       <c r="D63" s="163" t="s">
-        <v>71</v>
+        <v>143</v>
       </c>
       <c r="E63" s="163" t="s">
-        <v>148</v>
+        <v>61</v>
       </c>
       <c r="F63" s="341">
-        <v>2026</v>
+        <v>2023</v>
       </c>
       <c r="G63" s="164">
-        <v>46203</v>
+        <v>45583</v>
       </c>
       <c r="H63" s="164">
-        <v>46203</v>
+        <v>45583</v>
       </c>
       <c r="I63" s="161"/>
       <c r="J63" s="161"/>
@@ -9276,44 +9256,46 @@
         <v>562</v>
       </c>
       <c r="D64" s="163" t="s">
-        <v>143</v>
+        <v>71</v>
       </c>
       <c r="E64" s="163" t="s">
-        <v>61</v>
-      </c>
-      <c r="F64" s="341">
-        <v>2023</v>
-      </c>
-      <c r="G64" s="164">
-        <v>45583</v>
-      </c>
-      <c r="H64" s="164">
-        <v>45583</v>
-      </c>
+        <v>148</v>
+      </c>
+      <c r="F64" s="341"/>
+      <c r="G64" s="163"/>
+      <c r="H64" s="163"/>
       <c r="I64" s="161"/>
       <c r="J64" s="161"/>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A65" s="163" t="s">
-        <v>561</v>
+        <v>578</v>
       </c>
       <c r="B65" s="163" t="s">
-        <v>429</v>
+        <v>318</v>
       </c>
       <c r="C65" s="163" t="s">
-        <v>562</v>
+        <v>579</v>
       </c>
       <c r="D65" s="163" t="s">
-        <v>71</v>
+        <v>143</v>
       </c>
       <c r="E65" s="163" t="s">
-        <v>148</v>
-      </c>
-      <c r="F65" s="341"/>
-      <c r="G65" s="163"/>
-      <c r="H65" s="163"/>
-      <c r="I65" s="161"/>
-      <c r="J65" s="161"/>
+        <v>61</v>
+      </c>
+      <c r="F65" s="342">
+        <v>2020</v>
+      </c>
+      <c r="G65" s="126">
+        <v>43831</v>
+      </c>
+      <c r="H65" s="126">
+        <v>43831</v>
+      </c>
+      <c r="I65" s="124">
+        <v>20135</v>
+      </c>
+      <c r="J65" s="124"/>
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A66" s="163" t="s">
@@ -9326,52 +9308,49 @@
         <v>579</v>
       </c>
       <c r="D66" s="163" t="s">
+        <v>71</v>
+      </c>
+      <c r="E66" s="163" t="s">
+        <v>124</v>
+      </c>
+      <c r="F66" s="341" t="s">
+        <v>584</v>
+      </c>
+      <c r="G66" s="164">
+        <v>46203</v>
+      </c>
+      <c r="H66" s="164">
+        <v>46203</v>
+      </c>
+      <c r="I66" s="161"/>
+      <c r="J66" s="161"/>
+    </row>
+    <row r="67" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A67" s="105" t="s">
+        <v>590</v>
+      </c>
+      <c r="B67" s="163" t="s">
+        <v>435</v>
+      </c>
+      <c r="C67" s="163" t="s">
+        <v>591</v>
+      </c>
+      <c r="D67" s="163" t="s">
         <v>143</v>
       </c>
-      <c r="E66" s="163" t="s">
+      <c r="E67" s="163" t="s">
         <v>61</v>
       </c>
-      <c r="F66" s="342">
-        <v>2020</v>
-      </c>
-      <c r="G66" s="126">
-        <v>43831</v>
-      </c>
-      <c r="H66" s="126">
-        <v>43831</v>
-      </c>
-      <c r="I66" s="124">
-        <v>20135</v>
-      </c>
-      <c r="J66" s="124"/>
-    </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A67" s="163" t="s">
-        <v>578</v>
-      </c>
-      <c r="B67" s="163" t="s">
-        <v>318</v>
-      </c>
-      <c r="C67" s="163" t="s">
-        <v>579</v>
-      </c>
-      <c r="D67" s="163" t="s">
-        <v>71</v>
-      </c>
-      <c r="E67" s="163" t="s">
-        <v>124</v>
-      </c>
-      <c r="F67" s="341" t="s">
-        <v>584</v>
-      </c>
-      <c r="G67" s="164">
-        <v>46203</v>
-      </c>
-      <c r="H67" s="164">
-        <v>46203</v>
-      </c>
-      <c r="I67" s="161"/>
-      <c r="J67" s="161"/>
+      <c r="F67" s="342"/>
+      <c r="G67" s="126">
+        <v>44075</v>
+      </c>
+      <c r="H67" s="105"/>
+      <c r="I67" s="124">
+        <f>67243+12264</f>
+        <v>79507</v>
+      </c>
+      <c r="J67" s="124"/>
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A68" s="105" t="s">
@@ -9384,91 +9363,92 @@
         <v>591</v>
       </c>
       <c r="D68" s="163" t="s">
-        <v>143</v>
+        <v>71</v>
       </c>
       <c r="E68" s="163" t="s">
         <v>61</v>
       </c>
       <c r="F68" s="342"/>
-      <c r="G68" s="126">
-        <v>44075</v>
+      <c r="G68" s="242">
+        <v>45679</v>
       </c>
       <c r="H68" s="105"/>
-      <c r="I68" s="124">
-        <f>67243+12264</f>
-        <v>79507</v>
-      </c>
+      <c r="I68" s="124"/>
       <c r="J68" s="124"/>
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A69" s="105" t="s">
-        <v>590</v>
+      <c r="A69" s="163" t="s">
+        <v>602</v>
       </c>
       <c r="B69" s="163" t="s">
-        <v>435</v>
+        <v>603</v>
       </c>
       <c r="C69" s="163" t="s">
-        <v>591</v>
+        <v>604</v>
       </c>
       <c r="D69" s="163" t="s">
-        <v>71</v>
+        <v>214</v>
       </c>
       <c r="E69" s="163" t="s">
-        <v>61</v>
-      </c>
-      <c r="F69" s="342"/>
-      <c r="G69" s="242">
-        <v>45679</v>
-      </c>
-      <c r="H69" s="105"/>
-      <c r="I69" s="124"/>
-      <c r="J69" s="124"/>
+        <v>192</v>
+      </c>
+      <c r="F69" s="341" t="s">
+        <v>605</v>
+      </c>
+      <c r="G69" s="163"/>
+      <c r="H69" s="163"/>
+      <c r="I69" s="161"/>
+      <c r="J69" s="161"/>
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A70" s="163" t="s">
-        <v>602</v>
+        <v>1084</v>
       </c>
       <c r="B70" s="163" t="s">
-        <v>603</v>
+        <v>265</v>
       </c>
       <c r="C70" s="163" t="s">
-        <v>604</v>
-      </c>
-      <c r="D70" s="163" t="s">
-        <v>214</v>
-      </c>
-      <c r="E70" s="163" t="s">
-        <v>192</v>
-      </c>
-      <c r="F70" s="341" t="s">
-        <v>605</v>
-      </c>
-      <c r="G70" s="163"/>
-      <c r="H70" s="163"/>
-      <c r="I70" s="161"/>
-      <c r="J70" s="161"/>
+        <v>1083</v>
+      </c>
+      <c r="D70" s="163"/>
+      <c r="E70" s="163"/>
+      <c r="F70" s="341"/>
+      <c r="G70" s="126">
+        <v>45291</v>
+      </c>
+      <c r="H70" s="126">
+        <v>45291</v>
+      </c>
+      <c r="I70" s="161">
+        <v>33335</v>
+      </c>
+      <c r="J70" s="124"/>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A71" s="163" t="s">
-        <v>1084</v>
+        <v>613</v>
       </c>
       <c r="B71" s="163" t="s">
-        <v>265</v>
+        <v>58</v>
       </c>
       <c r="C71" s="163" t="s">
-        <v>1083</v>
-      </c>
-      <c r="D71" s="163"/>
-      <c r="E71" s="163"/>
-      <c r="F71" s="341"/>
+        <v>614</v>
+      </c>
+      <c r="D71" s="163" t="s">
+        <v>143</v>
+      </c>
+      <c r="E71" s="163" t="s">
+        <v>61</v>
+      </c>
+      <c r="F71" s="342">
+        <v>2020</v>
+      </c>
       <c r="G71" s="126">
-        <v>45291</v>
-      </c>
-      <c r="H71" s="126">
-        <v>45291</v>
-      </c>
-      <c r="I71" s="161">
-        <v>33335</v>
+        <v>43831</v>
+      </c>
+      <c r="H71" s="105"/>
+      <c r="I71" s="124">
+        <v>9653</v>
       </c>
       <c r="J71" s="124"/>
     </row>
@@ -9483,49 +9463,45 @@
         <v>614</v>
       </c>
       <c r="D72" s="163" t="s">
-        <v>143</v>
-      </c>
-      <c r="E72" s="163" t="s">
+        <v>71</v>
+      </c>
+      <c r="E72" s="105" t="s">
         <v>61</v>
       </c>
-      <c r="F72" s="342">
-        <v>2020</v>
+      <c r="F72" s="342" t="s">
+        <v>618</v>
       </c>
       <c r="G72" s="126">
-        <v>43831</v>
-      </c>
-      <c r="H72" s="105"/>
-      <c r="I72" s="124">
-        <v>9653</v>
-      </c>
-      <c r="J72" s="124"/>
+        <v>45536</v>
+      </c>
+      <c r="H72" s="126">
+        <v>45536</v>
+      </c>
+      <c r="I72" s="124"/>
+      <c r="J72" s="161"/>
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A73" s="163" t="s">
         <v>613</v>
       </c>
       <c r="B73" s="163" t="s">
-        <v>58</v>
+        <v>141</v>
       </c>
       <c r="C73" s="163" t="s">
-        <v>614</v>
+        <v>621</v>
       </c>
       <c r="D73" s="163" t="s">
         <v>71</v>
       </c>
-      <c r="E73" s="105" t="s">
+      <c r="E73" s="163" t="s">
         <v>61</v>
       </c>
-      <c r="F73" s="342" t="s">
-        <v>618</v>
-      </c>
-      <c r="G73" s="126">
-        <v>45536</v>
-      </c>
-      <c r="H73" s="126">
-        <v>45536</v>
-      </c>
-      <c r="I73" s="124"/>
+      <c r="F73" s="341"/>
+      <c r="G73" s="163"/>
+      <c r="H73" s="163"/>
+      <c r="I73" s="161">
+        <v>15000</v>
+      </c>
       <c r="J73" s="161"/>
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.2">
@@ -9539,39 +9515,43 @@
         <v>621</v>
       </c>
       <c r="D74" s="163" t="s">
-        <v>71</v>
+        <v>143</v>
       </c>
       <c r="E74" s="163" t="s">
-        <v>61</v>
+        <v>626</v>
       </c>
       <c r="F74" s="341"/>
       <c r="G74" s="163"/>
       <c r="H74" s="163"/>
-      <c r="I74" s="161">
-        <v>15000</v>
-      </c>
-      <c r="J74" s="161"/>
+      <c r="I74" s="161"/>
+      <c r="J74" s="124"/>
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A75" s="163" t="s">
         <v>613</v>
       </c>
       <c r="B75" s="163" t="s">
-        <v>141</v>
-      </c>
-      <c r="C75" s="163" t="s">
-        <v>621</v>
+        <v>444</v>
+      </c>
+      <c r="C75" s="328" t="s">
+        <v>628</v>
       </c>
       <c r="D75" s="163" t="s">
         <v>143</v>
       </c>
       <c r="E75" s="163" t="s">
-        <v>626</v>
-      </c>
-      <c r="F75" s="341"/>
-      <c r="G75" s="163"/>
-      <c r="H75" s="163"/>
-      <c r="I75" s="161"/>
+        <v>192</v>
+      </c>
+      <c r="F75" s="342"/>
+      <c r="G75" s="126">
+        <v>43559</v>
+      </c>
+      <c r="H75" s="126">
+        <v>43559</v>
+      </c>
+      <c r="I75" s="124">
+        <v>49264</v>
+      </c>
       <c r="J75" s="124"/>
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.2">
@@ -9585,21 +9565,21 @@
         <v>628</v>
       </c>
       <c r="D76" s="163" t="s">
-        <v>143</v>
+        <v>71</v>
       </c>
       <c r="E76" s="163" t="s">
-        <v>192</v>
-      </c>
-      <c r="F76" s="342"/>
+        <v>148</v>
+      </c>
+      <c r="F76" s="342">
+        <v>2023</v>
+      </c>
       <c r="G76" s="126">
-        <v>43559</v>
+        <v>45107</v>
       </c>
       <c r="H76" s="126">
-        <v>43559</v>
-      </c>
-      <c r="I76" s="124">
-        <v>49264</v>
-      </c>
+        <v>45108</v>
+      </c>
+      <c r="I76" s="124"/>
       <c r="J76" s="124"/>
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.2">
@@ -9607,27 +9587,29 @@
         <v>613</v>
       </c>
       <c r="B77" s="163" t="s">
-        <v>444</v>
-      </c>
-      <c r="C77" s="328" t="s">
-        <v>628</v>
+        <v>318</v>
+      </c>
+      <c r="C77" s="105" t="s">
+        <v>638</v>
       </c>
       <c r="D77" s="163" t="s">
-        <v>71</v>
+        <v>143</v>
       </c>
       <c r="E77" s="163" t="s">
-        <v>148</v>
+        <v>61</v>
       </c>
       <c r="F77" s="342">
-        <v>2023</v>
+        <v>2012</v>
       </c>
       <c r="G77" s="126">
-        <v>45107</v>
+        <v>41061</v>
       </c>
       <c r="H77" s="126">
-        <v>45108</v>
-      </c>
-      <c r="I77" s="124"/>
+        <v>41061</v>
+      </c>
+      <c r="I77" s="124">
+        <v>3734</v>
+      </c>
       <c r="J77" s="124"/>
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.2">
@@ -9641,23 +9623,21 @@
         <v>638</v>
       </c>
       <c r="D78" s="163" t="s">
-        <v>143</v>
+        <v>71</v>
       </c>
       <c r="E78" s="163" t="s">
         <v>61</v>
       </c>
-      <c r="F78" s="342">
-        <v>2012</v>
+      <c r="F78" s="342" t="s">
+        <v>511</v>
       </c>
       <c r="G78" s="126">
-        <v>41061</v>
+        <v>44501</v>
       </c>
       <c r="H78" s="126">
-        <v>41061</v>
-      </c>
-      <c r="I78" s="124">
-        <v>3734</v>
-      </c>
+        <v>44502</v>
+      </c>
+      <c r="I78" s="124"/>
       <c r="J78" s="124"/>
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.2">
@@ -9674,17 +9654,11 @@
         <v>71</v>
       </c>
       <c r="E79" s="163" t="s">
-        <v>61</v>
-      </c>
-      <c r="F79" s="342" t="s">
-        <v>511</v>
-      </c>
-      <c r="G79" s="126">
-        <v>44501</v>
-      </c>
-      <c r="H79" s="126">
-        <v>44502</v>
-      </c>
+        <v>124</v>
+      </c>
+      <c r="F79" s="342"/>
+      <c r="G79" s="105"/>
+      <c r="H79" s="105"/>
       <c r="I79" s="124"/>
       <c r="J79" s="124"/>
     </row>
@@ -9695,47 +9669,53 @@
       <c r="B80" s="163" t="s">
         <v>318</v>
       </c>
-      <c r="C80" s="105" t="s">
-        <v>638</v>
+      <c r="C80" s="163" t="s">
+        <v>649</v>
       </c>
       <c r="D80" s="163" t="s">
-        <v>71</v>
+        <v>143</v>
       </c>
       <c r="E80" s="163" t="s">
         <v>124</v>
       </c>
-      <c r="F80" s="342"/>
-      <c r="G80" s="105"/>
-      <c r="H80" s="105"/>
+      <c r="F80" s="344">
+        <v>46508</v>
+      </c>
+      <c r="G80" s="126">
+        <v>46508</v>
+      </c>
+      <c r="H80" s="126">
+        <v>46508</v>
+      </c>
       <c r="I80" s="124"/>
       <c r="J80" s="124"/>
     </row>
     <row r="81" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A81" s="163" t="s">
-        <v>613</v>
+        <v>652</v>
       </c>
       <c r="B81" s="163" t="s">
-        <v>318</v>
+        <v>265</v>
       </c>
       <c r="C81" s="163" t="s">
-        <v>649</v>
+        <v>653</v>
       </c>
       <c r="D81" s="163" t="s">
         <v>143</v>
       </c>
       <c r="E81" s="163" t="s">
-        <v>124</v>
-      </c>
-      <c r="F81" s="344">
-        <v>46508</v>
-      </c>
+        <v>61</v>
+      </c>
+      <c r="F81" s="342"/>
       <c r="G81" s="126">
-        <v>46508</v>
+        <v>45291</v>
       </c>
       <c r="H81" s="126">
-        <v>46508</v>
-      </c>
-      <c r="I81" s="124"/>
+        <v>45291</v>
+      </c>
+      <c r="I81" s="124">
+        <v>42533</v>
+      </c>
       <c r="J81" s="124"/>
     </row>
     <row r="82" spans="1:10" x14ac:dyDescent="0.2">
@@ -9745,14 +9725,14 @@
       <c r="B82" s="163" t="s">
         <v>265</v>
       </c>
-      <c r="C82" s="163" t="s">
-        <v>653</v>
+      <c r="C82" s="138" t="s">
+        <v>657</v>
       </c>
       <c r="D82" s="163" t="s">
         <v>143</v>
       </c>
       <c r="E82" s="163" t="s">
-        <v>61</v>
+        <v>148</v>
       </c>
       <c r="F82" s="342"/>
       <c r="G82" s="126">
@@ -9762,7 +9742,7 @@
         <v>45291</v>
       </c>
       <c r="I82" s="124">
-        <v>42533</v>
+        <v>15433</v>
       </c>
       <c r="J82" s="124"/>
     </row>
@@ -9774,42 +9754,38 @@
         <v>265</v>
       </c>
       <c r="C83" s="138" t="s">
-        <v>657</v>
+        <v>663</v>
       </c>
       <c r="D83" s="163" t="s">
-        <v>143</v>
+        <v>214</v>
       </c>
       <c r="E83" s="163" t="s">
-        <v>148</v>
+        <v>61</v>
       </c>
       <c r="F83" s="342"/>
       <c r="G83" s="126">
-        <v>45291</v>
+        <v>45657</v>
       </c>
       <c r="H83" s="126">
-        <v>45291</v>
+        <v>45657</v>
       </c>
       <c r="I83" s="124">
-        <v>15433</v>
+        <v>24008</v>
       </c>
       <c r="J83" s="124"/>
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A84" s="163" t="s">
-        <v>652</v>
+        <v>667</v>
       </c>
       <c r="B84" s="163" t="s">
         <v>265</v>
       </c>
-      <c r="C84" s="138" t="s">
-        <v>663</v>
-      </c>
-      <c r="D84" s="163" t="s">
-        <v>214</v>
-      </c>
-      <c r="E84" s="163" t="s">
-        <v>61</v>
-      </c>
+      <c r="C84" s="163" t="s">
+        <v>668</v>
+      </c>
+      <c r="D84" s="163"/>
+      <c r="E84" s="163"/>
       <c r="F84" s="342"/>
       <c r="G84" s="126">
         <v>45657</v>
@@ -9818,7 +9794,7 @@
         <v>45657</v>
       </c>
       <c r="I84" s="124">
-        <v>24008</v>
+        <v>23534</v>
       </c>
       <c r="J84" s="124"/>
     </row>
@@ -9832,17 +9808,15 @@
       <c r="C85" s="163" t="s">
         <v>668</v>
       </c>
-      <c r="D85" s="163"/>
-      <c r="E85" s="163"/>
-      <c r="F85" s="342"/>
-      <c r="G85" s="126">
-        <v>45657</v>
-      </c>
-      <c r="H85" s="126">
-        <v>45657</v>
-      </c>
-      <c r="I85" s="124">
-        <v>23534</v>
+      <c r="D85" s="163" t="s">
+        <v>143</v>
+      </c>
+      <c r="E85" s="163" t="s">
+        <v>61</v>
+      </c>
+      <c r="F85" s="341"/>
+      <c r="I85" s="161">
+        <v>5000</v>
       </c>
       <c r="J85" s="124"/>
     </row>
@@ -9851,10 +9825,10 @@
         <v>667</v>
       </c>
       <c r="B86" s="163" t="s">
-        <v>265</v>
+        <v>182</v>
       </c>
       <c r="C86" s="163" t="s">
-        <v>668</v>
+        <v>680</v>
       </c>
       <c r="D86" s="163" t="s">
         <v>143</v>
@@ -9862,21 +9836,25 @@
       <c r="E86" s="163" t="s">
         <v>61</v>
       </c>
-      <c r="F86" s="341"/>
+      <c r="F86" s="341" t="s">
+        <v>682</v>
+      </c>
+      <c r="G86" s="163"/>
+      <c r="H86" s="163"/>
       <c r="I86" s="161">
-        <v>5000</v>
-      </c>
-      <c r="J86" s="124"/>
+        <v>111872</v>
+      </c>
+      <c r="J86" s="161"/>
     </row>
     <row r="87" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A87" s="163" t="s">
         <v>667</v>
       </c>
       <c r="B87" s="163" t="s">
-        <v>182</v>
+        <v>357</v>
       </c>
       <c r="C87" s="163" t="s">
-        <v>680</v>
+        <v>691</v>
       </c>
       <c r="D87" s="163" t="s">
         <v>143</v>
@@ -9885,66 +9863,70 @@
         <v>61</v>
       </c>
       <c r="F87" s="341" t="s">
-        <v>682</v>
+        <v>694</v>
       </c>
       <c r="G87" s="163"/>
       <c r="H87" s="163"/>
-      <c r="I87" s="161">
-        <v>111872</v>
-      </c>
+      <c r="I87" s="161"/>
       <c r="J87" s="161"/>
     </row>
     <row r="88" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A88" s="163" t="s">
-        <v>667</v>
-      </c>
-      <c r="B88" s="163" t="s">
-        <v>357</v>
-      </c>
-      <c r="C88" s="163" t="s">
-        <v>691</v>
-      </c>
-      <c r="D88" s="163" t="s">
+      <c r="A88" s="183" t="s">
+        <v>703</v>
+      </c>
+      <c r="B88" s="183" t="s">
+        <v>704</v>
+      </c>
+      <c r="C88" s="183" t="s">
+        <v>705</v>
+      </c>
+      <c r="D88" s="183" t="s">
         <v>143</v>
       </c>
-      <c r="E88" s="163" t="s">
+      <c r="E88" s="183" t="s">
         <v>61</v>
       </c>
-      <c r="F88" s="341" t="s">
-        <v>694</v>
-      </c>
-      <c r="G88" s="163"/>
-      <c r="H88" s="163"/>
-      <c r="I88" s="161"/>
-      <c r="J88" s="161"/>
+      <c r="F88" s="342" t="s">
+        <v>708</v>
+      </c>
+      <c r="G88" s="126">
+        <v>46023</v>
+      </c>
+      <c r="H88" s="126">
+        <v>46023</v>
+      </c>
+      <c r="I88" s="124">
+        <v>50000</v>
+      </c>
+      <c r="J88" s="124"/>
     </row>
     <row r="89" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A89" s="183" t="s">
-        <v>703</v>
-      </c>
-      <c r="B89" s="183" t="s">
-        <v>704</v>
-      </c>
-      <c r="C89" s="183" t="s">
-        <v>705</v>
-      </c>
-      <c r="D89" s="183" t="s">
+      <c r="A89" s="163" t="s">
+        <v>1028</v>
+      </c>
+      <c r="B89" s="163" t="s">
+        <v>141</v>
+      </c>
+      <c r="C89" s="163" t="s">
+        <v>1029</v>
+      </c>
+      <c r="D89" s="163" t="s">
         <v>143</v>
       </c>
-      <c r="E89" s="183" t="s">
+      <c r="E89" s="163" t="s">
         <v>61</v>
       </c>
-      <c r="F89" s="342" t="s">
-        <v>708</v>
-      </c>
-      <c r="G89" s="126">
-        <v>46023</v>
-      </c>
-      <c r="H89" s="126">
-        <v>46023</v>
-      </c>
-      <c r="I89" s="124">
-        <v>50000</v>
+      <c r="F89" s="341">
+        <v>2018</v>
+      </c>
+      <c r="G89" s="164">
+        <v>43101</v>
+      </c>
+      <c r="H89" s="164">
+        <v>43101</v>
+      </c>
+      <c r="I89" s="161">
+        <v>14287</v>
       </c>
       <c r="J89" s="124"/>
     </row>
@@ -9959,24 +9941,18 @@
         <v>1029</v>
       </c>
       <c r="D90" s="163" t="s">
-        <v>143</v>
+        <v>71</v>
       </c>
       <c r="E90" s="163" t="s">
         <v>61</v>
       </c>
-      <c r="F90" s="341">
-        <v>2018</v>
-      </c>
-      <c r="G90" s="164">
-        <v>43101</v>
-      </c>
-      <c r="H90" s="164">
-        <v>43101</v>
-      </c>
+      <c r="F90" s="341"/>
+      <c r="G90" s="164"/>
+      <c r="H90" s="164"/>
       <c r="I90" s="161">
-        <v>14287</v>
-      </c>
-      <c r="J90" s="124"/>
+        <v>10881</v>
+      </c>
+      <c r="J90" s="161"/>
     </row>
     <row r="91" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A91" s="163" t="s">
@@ -9991,150 +9967,150 @@
       <c r="D91" s="163" t="s">
         <v>71</v>
       </c>
-      <c r="E91" s="163" t="s">
-        <v>61</v>
+      <c r="E91" s="105" t="s">
+        <v>148</v>
       </c>
       <c r="F91" s="341"/>
-      <c r="G91" s="164"/>
-      <c r="H91" s="164"/>
-      <c r="I91" s="161">
-        <v>10881</v>
-      </c>
+      <c r="G91" s="163"/>
+      <c r="H91" s="163"/>
+      <c r="I91" s="161"/>
       <c r="J91" s="161"/>
     </row>
     <row r="92" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A92" s="163" t="s">
-        <v>1028</v>
+        <v>718</v>
       </c>
       <c r="B92" s="163" t="s">
-        <v>141</v>
+        <v>58</v>
       </c>
       <c r="C92" s="163" t="s">
-        <v>1029</v>
+        <v>375</v>
       </c>
       <c r="D92" s="163" t="s">
-        <v>71</v>
-      </c>
-      <c r="E92" s="105" t="s">
-        <v>148</v>
-      </c>
-      <c r="F92" s="341"/>
-      <c r="G92" s="163"/>
-      <c r="H92" s="163"/>
-      <c r="I92" s="161"/>
-      <c r="J92" s="161"/>
+        <v>143</v>
+      </c>
+      <c r="E92" s="163" t="s">
+        <v>61</v>
+      </c>
+      <c r="F92" s="341" t="s">
+        <v>721</v>
+      </c>
+      <c r="G92" s="164">
+        <v>44642</v>
+      </c>
+      <c r="H92" s="164">
+        <v>44642</v>
+      </c>
+      <c r="I92" s="124">
+        <v>206097</v>
+      </c>
+      <c r="J92" s="124"/>
     </row>
     <row r="93" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A93" s="163" t="s">
         <v>718</v>
       </c>
       <c r="B93" s="163" t="s">
-        <v>58</v>
+        <v>335</v>
       </c>
       <c r="C93" s="163" t="s">
-        <v>375</v>
+        <v>729</v>
       </c>
       <c r="D93" s="163" t="s">
         <v>143</v>
       </c>
       <c r="E93" s="163" t="s">
-        <v>61</v>
-      </c>
-      <c r="F93" s="341" t="s">
-        <v>721</v>
+        <v>192</v>
+      </c>
+      <c r="F93" s="341">
+        <v>2015</v>
       </c>
       <c r="G93" s="164">
-        <v>44642</v>
+        <v>42156</v>
       </c>
       <c r="H93" s="164">
-        <v>44642</v>
-      </c>
-      <c r="I93" s="124">
-        <v>206097</v>
-      </c>
-      <c r="J93" s="124"/>
+        <v>42157</v>
+      </c>
+      <c r="I93" s="161"/>
+      <c r="J93" s="161"/>
     </row>
     <row r="94" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A94" s="163" t="s">
-        <v>718</v>
+        <v>737</v>
       </c>
       <c r="B94" s="163" t="s">
-        <v>335</v>
+        <v>212</v>
       </c>
       <c r="C94" s="163" t="s">
-        <v>729</v>
+        <v>738</v>
       </c>
       <c r="D94" s="163" t="s">
         <v>143</v>
       </c>
       <c r="E94" s="163" t="s">
-        <v>192</v>
-      </c>
-      <c r="F94" s="341">
-        <v>2015</v>
-      </c>
-      <c r="G94" s="164">
-        <v>42156</v>
-      </c>
-      <c r="H94" s="164">
-        <v>42157</v>
-      </c>
-      <c r="I94" s="161"/>
+        <v>148</v>
+      </c>
+      <c r="F94" s="341" t="s">
+        <v>739</v>
+      </c>
+      <c r="G94" s="163"/>
+      <c r="H94" s="163"/>
+      <c r="I94" s="161">
+        <v>30000</v>
+      </c>
       <c r="J94" s="161"/>
     </row>
     <row r="95" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A95" s="163" t="s">
-        <v>737</v>
-      </c>
-      <c r="B95" s="163" t="s">
-        <v>212</v>
-      </c>
-      <c r="C95" s="163" t="s">
-        <v>738</v>
-      </c>
-      <c r="D95" s="163" t="s">
+      <c r="A95" s="183" t="s">
+        <v>575</v>
+      </c>
+      <c r="B95" s="183" t="s">
+        <v>444</v>
+      </c>
+      <c r="C95" s="183" t="s">
+        <v>745</v>
+      </c>
+      <c r="D95" s="183" t="s">
         <v>143</v>
       </c>
-      <c r="E95" s="163" t="s">
-        <v>148</v>
-      </c>
-      <c r="F95" s="341" t="s">
-        <v>739</v>
-      </c>
-      <c r="G95" s="163"/>
-      <c r="H95" s="163"/>
-      <c r="I95" s="161">
-        <v>30000</v>
+      <c r="E95" s="183" t="s">
+        <v>61</v>
+      </c>
+      <c r="F95" s="342">
+        <v>2013</v>
+      </c>
+      <c r="G95" s="126">
+        <v>41426</v>
+      </c>
+      <c r="H95" s="126">
+        <v>41426</v>
+      </c>
+      <c r="I95" s="124">
+        <v>94839</v>
       </c>
       <c r="J95" s="161"/>
     </row>
     <row r="96" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A96" s="183" t="s">
+      <c r="A96" s="163" t="s">
         <v>575</v>
       </c>
-      <c r="B96" s="183" t="s">
-        <v>444</v>
-      </c>
-      <c r="C96" s="183" t="s">
-        <v>745</v>
-      </c>
-      <c r="D96" s="183" t="s">
-        <v>143</v>
-      </c>
-      <c r="E96" s="183" t="s">
+      <c r="B96" s="163" t="s">
+        <v>58</v>
+      </c>
+      <c r="C96" s="163" t="s">
+        <v>754</v>
+      </c>
+      <c r="D96" s="163" t="s">
+        <v>214</v>
+      </c>
+      <c r="E96" s="163" t="s">
         <v>61</v>
       </c>
-      <c r="F96" s="342">
-        <v>2013</v>
-      </c>
-      <c r="G96" s="126">
-        <v>41426</v>
-      </c>
-      <c r="H96" s="126">
-        <v>41426</v>
-      </c>
-      <c r="I96" s="124">
-        <v>94839</v>
+      <c r="F96" s="341"/>
+      <c r="G96" s="163"/>
+      <c r="H96" s="163"/>
+      <c r="I96" s="161">
+        <v>140000</v>
       </c>
       <c r="J96" s="161"/>
     </row>
@@ -10146,7 +10122,7 @@
         <v>58</v>
       </c>
       <c r="C97" s="163" t="s">
-        <v>754</v>
+        <v>764</v>
       </c>
       <c r="D97" s="163" t="s">
         <v>214</v>
@@ -10158,7 +10134,7 @@
       <c r="G97" s="163"/>
       <c r="H97" s="163"/>
       <c r="I97" s="161">
-        <v>140000</v>
+        <v>15000</v>
       </c>
       <c r="J97" s="161"/>
     </row>
@@ -10170,20 +10146,20 @@
         <v>58</v>
       </c>
       <c r="C98" s="163" t="s">
-        <v>764</v>
+        <v>770</v>
       </c>
       <c r="D98" s="163" t="s">
-        <v>214</v>
+        <v>143</v>
       </c>
       <c r="E98" s="163" t="s">
-        <v>61</v>
-      </c>
-      <c r="F98" s="341"/>
+        <v>192</v>
+      </c>
+      <c r="F98" s="341" t="s">
+        <v>772</v>
+      </c>
       <c r="G98" s="163"/>
       <c r="H98" s="163"/>
-      <c r="I98" s="161">
-        <v>15000</v>
-      </c>
+      <c r="I98" s="161"/>
       <c r="J98" s="161"/>
     </row>
     <row r="99" spans="1:10" x14ac:dyDescent="0.2">
@@ -10194,20 +10170,26 @@
         <v>58</v>
       </c>
       <c r="C99" s="163" t="s">
-        <v>770</v>
+        <v>781</v>
       </c>
       <c r="D99" s="163" t="s">
-        <v>143</v>
-      </c>
-      <c r="E99" s="163" t="s">
-        <v>192</v>
+        <v>214</v>
+      </c>
+      <c r="E99" s="206" t="s">
+        <v>61</v>
       </c>
       <c r="F99" s="341" t="s">
-        <v>772</v>
-      </c>
-      <c r="G99" s="163"/>
-      <c r="H99" s="163"/>
-      <c r="I99" s="161"/>
+        <v>782</v>
+      </c>
+      <c r="G99" s="164">
+        <v>43773</v>
+      </c>
+      <c r="H99" s="164">
+        <v>43773</v>
+      </c>
+      <c r="I99" s="161">
+        <v>333000</v>
+      </c>
       <c r="J99" s="161"/>
     </row>
     <row r="100" spans="1:10" x14ac:dyDescent="0.2">
@@ -10215,95 +10197,93 @@
         <v>575</v>
       </c>
       <c r="B100" s="163" t="s">
-        <v>58</v>
+        <v>318</v>
       </c>
       <c r="C100" s="163" t="s">
-        <v>781</v>
+        <v>792</v>
       </c>
       <c r="D100" s="163" t="s">
-        <v>214</v>
-      </c>
-      <c r="E100" s="206" t="s">
-        <v>61</v>
-      </c>
-      <c r="F100" s="341" t="s">
-        <v>782</v>
+        <v>143</v>
+      </c>
+      <c r="E100" s="163" t="s">
+        <v>148</v>
+      </c>
+      <c r="F100" s="341">
+        <v>2025</v>
       </c>
       <c r="G100" s="164">
-        <v>43773</v>
-      </c>
-      <c r="H100" s="164">
-        <v>43773</v>
-      </c>
+        <v>45809</v>
+      </c>
+      <c r="H100" s="163"/>
       <c r="I100" s="161">
-        <v>333000</v>
+        <f>3000000/5</f>
+        <v>600000</v>
       </c>
       <c r="J100" s="161"/>
     </row>
     <row r="101" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A101" s="163" t="s">
-        <v>575</v>
+        <v>824</v>
       </c>
       <c r="B101" s="163" t="s">
-        <v>318</v>
+        <v>825</v>
       </c>
       <c r="C101" s="163" t="s">
-        <v>792</v>
-      </c>
-      <c r="D101" s="163" t="s">
-        <v>143</v>
+        <v>826</v>
+      </c>
+      <c r="D101" s="105" t="s">
+        <v>60</v>
       </c>
       <c r="E101" s="163" t="s">
         <v>148</v>
       </c>
-      <c r="F101" s="341">
-        <v>2025</v>
-      </c>
-      <c r="G101" s="164">
-        <v>45809</v>
-      </c>
-      <c r="H101" s="163"/>
-      <c r="I101" s="161">
-        <f>3000000/5</f>
-        <v>600000</v>
-      </c>
-      <c r="J101" s="161"/>
+      <c r="F101" s="342"/>
+      <c r="G101" s="105"/>
+      <c r="H101" s="126">
+        <v>45717</v>
+      </c>
+      <c r="I101" s="124">
+        <v>85654</v>
+      </c>
+      <c r="J101" s="124"/>
     </row>
     <row r="102" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A102" s="163" t="s">
-        <v>824</v>
+        <v>810</v>
       </c>
       <c r="B102" s="163" t="s">
-        <v>825</v>
+        <v>265</v>
       </c>
       <c r="C102" s="163" t="s">
-        <v>826</v>
-      </c>
-      <c r="D102" s="105" t="s">
-        <v>60</v>
+        <v>811</v>
+      </c>
+      <c r="D102" s="163" t="s">
+        <v>143</v>
       </c>
       <c r="E102" s="163" t="s">
-        <v>148</v>
-      </c>
-      <c r="F102" s="342"/>
-      <c r="G102" s="105"/>
-      <c r="H102" s="126">
-        <v>45717</v>
-      </c>
-      <c r="I102" s="124">
-        <v>85654</v>
-      </c>
-      <c r="J102" s="124"/>
+        <v>61</v>
+      </c>
+      <c r="F102" s="341">
+        <v>2019</v>
+      </c>
+      <c r="G102" s="164">
+        <v>43646</v>
+      </c>
+      <c r="H102" s="164">
+        <v>43646</v>
+      </c>
+      <c r="I102" s="161"/>
+      <c r="J102" s="161"/>
     </row>
     <row r="103" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A103" s="163" t="s">
         <v>810</v>
       </c>
       <c r="B103" s="163" t="s">
-        <v>265</v>
+        <v>212</v>
       </c>
       <c r="C103" s="163" t="s">
-        <v>811</v>
+        <v>817</v>
       </c>
       <c r="D103" s="163" t="s">
         <v>143</v>
@@ -10311,14 +10291,12 @@
       <c r="E103" s="163" t="s">
         <v>61</v>
       </c>
-      <c r="F103" s="341">
-        <v>2019</v>
-      </c>
+      <c r="F103" s="341"/>
       <c r="G103" s="164">
-        <v>43646</v>
+        <v>45183</v>
       </c>
       <c r="H103" s="164">
-        <v>43646</v>
+        <v>45183</v>
       </c>
       <c r="I103" s="161"/>
       <c r="J103" s="161"/>
@@ -10334,99 +10312,73 @@
         <v>817</v>
       </c>
       <c r="D104" s="163" t="s">
-        <v>143</v>
+        <v>71</v>
       </c>
       <c r="E104" s="163" t="s">
-        <v>61</v>
+        <v>148</v>
       </c>
       <c r="F104" s="341"/>
       <c r="G104" s="164">
-        <v>45183</v>
+        <v>45777</v>
       </c>
       <c r="H104" s="164">
-        <v>45183</v>
+        <v>45777</v>
       </c>
       <c r="I104" s="161"/>
       <c r="J104" s="161"/>
     </row>
     <row r="105" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A105" s="163" t="s">
-        <v>810</v>
+        <v>839</v>
       </c>
       <c r="B105" s="163" t="s">
-        <v>212</v>
+        <v>58</v>
       </c>
       <c r="C105" s="163" t="s">
-        <v>817</v>
+        <v>840</v>
       </c>
       <c r="D105" s="163" t="s">
-        <v>71</v>
+        <v>143</v>
       </c>
       <c r="E105" s="163" t="s">
-        <v>148</v>
+        <v>192</v>
       </c>
       <c r="F105" s="341"/>
-      <c r="G105" s="164">
-        <v>45777</v>
-      </c>
-      <c r="H105" s="164">
-        <v>45777</v>
-      </c>
+      <c r="G105" s="163"/>
+      <c r="H105" s="163"/>
       <c r="I105" s="161"/>
       <c r="J105" s="161"/>
     </row>
     <row r="106" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A106" s="163" t="s">
-        <v>839</v>
+        <v>847</v>
       </c>
       <c r="B106" s="163" t="s">
-        <v>58</v>
+        <v>444</v>
       </c>
       <c r="C106" s="163" t="s">
-        <v>840</v>
+        <v>802</v>
       </c>
       <c r="D106" s="163" t="s">
         <v>143</v>
       </c>
       <c r="E106" s="163" t="s">
-        <v>192</v>
+        <v>626</v>
       </c>
       <c r="F106" s="341"/>
       <c r="G106" s="163"/>
       <c r="H106" s="163"/>
-      <c r="I106" s="161"/>
+      <c r="I106" s="161">
+        <v>60000</v>
+      </c>
       <c r="J106" s="161"/>
     </row>
     <row r="107" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A107" s="163" t="s">
-        <v>847</v>
-      </c>
-      <c r="B107" s="163" t="s">
-        <v>444</v>
-      </c>
-      <c r="C107" s="163" t="s">
-        <v>802</v>
-      </c>
-      <c r="D107" s="163" t="s">
-        <v>143</v>
-      </c>
-      <c r="E107" s="163" t="s">
-        <v>626</v>
-      </c>
-      <c r="F107" s="341"/>
-      <c r="G107" s="163"/>
-      <c r="H107" s="163"/>
-      <c r="I107" s="161">
-        <v>60000</v>
-      </c>
-      <c r="J107" s="161"/>
-    </row>
-    <row r="108" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A108" s="163"/>
-      <c r="B108" s="163"/>
-      <c r="C108" s="163"/>
-      <c r="D108" s="163"/>
-      <c r="E108" s="163"/>
+      <c r="A107" s="163"/>
+      <c r="B107" s="163"/>
+      <c r="C107" s="163"/>
+      <c r="D107" s="163"/>
+      <c r="E107" s="163"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -37978,6 +37930,51 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <ProjectType xmlns="a800b4a7-713e-40fb-b259-074d23fe1c46">
+      <Value>Dataset</Value>
+    </ProjectType>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a800b4a7-713e-40fb-b259-074d23fe1c46">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <ResearchArea xmlns="a800b4a7-713e-40fb-b259-074d23fe1c46">
+      <Value>Green Economy</Value>
+    </ResearchArea>
+    <TaxCatchAll xmlns="b17ea8e4-3fb0-4555-9c20-069a19b46cb2" xsi:nil="true"/>
+    <FinalTitle xmlns="a800b4a7-713e-40fb-b259-074d23fe1c46" xsi:nil="true"/>
+    <LinktoPublication xmlns="a800b4a7-713e-40fb-b259-074d23fe1c46" xsi:nil="true"/>
+    <Authors xmlns="b17ea8e4-3fb0-4555-9c20-069a19b46cb2">
+      <UserInfo>
+        <DisplayName>Ugne Keliauskaite</DisplayName>
+        <AccountId>1048</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Ben McWilliams</DisplayName>
+        <AccountId>22</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Marie Jugé</DisplayName>
+        <AccountId>1714</AccountId>
+        <AccountType/>
+      </UserInfo>
+    </Authors>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005608FA096EBB4B4B8A364436FE5AF333" ma:contentTypeVersion="22" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="14f258b733f6365362ddc6ad739ca240">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b17ea8e4-3fb0-4555-9c20-069a19b46cb2" xmlns:ns3="a800b4a7-713e-40fb-b259-074d23fe1c46" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="392726fe05a3a4dbab19059d5b4c5bb0" ns2:_="" ns3:_="">
     <xsd:import namespace="b17ea8e4-3fb0-4555-9c20-069a19b46cb2"/>
@@ -38310,66 +38307,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <ProjectType xmlns="a800b4a7-713e-40fb-b259-074d23fe1c46">
-      <Value>Dataset</Value>
-    </ProjectType>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a800b4a7-713e-40fb-b259-074d23fe1c46">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <ResearchArea xmlns="a800b4a7-713e-40fb-b259-074d23fe1c46">
-      <Value>Green Economy</Value>
-    </ResearchArea>
-    <TaxCatchAll xmlns="b17ea8e4-3fb0-4555-9c20-069a19b46cb2" xsi:nil="true"/>
-    <FinalTitle xmlns="a800b4a7-713e-40fb-b259-074d23fe1c46" xsi:nil="true"/>
-    <LinktoPublication xmlns="a800b4a7-713e-40fb-b259-074d23fe1c46" xsi:nil="true"/>
-    <Authors xmlns="b17ea8e4-3fb0-4555-9c20-069a19b46cb2">
-      <UserInfo>
-        <DisplayName>Ugne Keliauskaite</DisplayName>
-        <AccountId>1048</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Ben McWilliams</DisplayName>
-        <AccountId>22</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Marie Jugé</DisplayName>
-        <AccountId>1714</AccountId>
-        <AccountType/>
-      </UserInfo>
-    </Authors>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD7AB568-E6EA-474D-8278-D37477DAFA72}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8781AB9E-9F28-4A8F-99EF-C45B15DD4F97}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="b17ea8e4-3fb0-4555-9c20-069a19b46cb2"/>
-    <ds:schemaRef ds:uri="a800b4a7-713e-40fb-b259-074d23fe1c46"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -38392,9 +38333,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8781AB9E-9F28-4A8F-99EF-C45B15DD4F97}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD7AB568-E6EA-474D-8278-D37477DAFA72}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="b17ea8e4-3fb0-4555-9c20-069a19b46cb2"/>
+    <ds:schemaRef ds:uri="a800b4a7-713e-40fb-b259-074d23fe1c46"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>